<commit_message>
Keep local Vercel env files out of git, and publish the latest nutrition sheets and page data versions.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Product-nutritional-ingredients-data/C014W C014WE -1L Gluten Free Reduced Salt Soy Sauce without vinegar.xlsx
+++ b/Product-nutritional-ingredients-data/C014W C014WE -1L Gluten Free Reduced Salt Soy Sauce without vinegar.xlsx
@@ -6511,19 +6511,19 @@
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3bb59413-afb5-4b9b-85e8-61d2b74a5666">
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e3d68449-7656-4e01-bff5-0ba578631d01">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4faae966-7260-43d3-ae92-efca4c8c38c2" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4e3da3af-ee5c-4759-aab6-a01dc2b41ec5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A19C90FBB319384E9453BC654633A1BE" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f12f626cb4656acfa57bc6e2f51cc2d0">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3bb59413-afb5-4b9b-85e8-61d2b74a5666" xmlns:ns3="4faae966-7260-43d3-ae92-efca4c8c38c2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="893be911098693cceb085112851dd985" ns2:_="" ns3:_="">
-    <xsd:import namespace="3bb59413-afb5-4b9b-85e8-61d2b74a5666"/>
-    <xsd:import namespace="4faae966-7260-43d3-ae92-efca4c8c38c2"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008D5A50B03D5E3D4C9F83ADD28043CA33" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4b8a87e1fee6cea9982f2ac75f1afdf">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e3d68449-7656-4e01-bff5-0ba578631d01" xmlns:ns3="4e3da3af-ee5c-4759-aab6-a01dc2b41ec5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="59e937c2640ac7e7f487c2c3bc7ea16a" ns2:_="" ns3:_="">
+    <xsd:import namespace="e3d68449-7656-4e01-bff5-0ba578631d01"/>
+    <xsd:import namespace="4e3da3af-ee5c-4759-aab6-a01dc2b41ec5"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -6532,21 +6532,17 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
                 <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -6554,7 +6550,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="3bb59413-afb5-4b9b-85e8-61d2b74a5666" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e3d68449-7656-4e01-bff5-0ba578631d01" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -6567,103 +6563,65 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceAutoTags" ma:index="11" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="12" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="22" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="a42d9c68-cab4-4c2b-b9bf-2edd401046ce" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="a42d9c68-cab4-4c2b-b9bf-2edd401046ce" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="19" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="20" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="4faae966-7260-43d3-ae92-efca4c8c38c2" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="4e3da3af-ee5c-4759-aab6-a01dc2b41ec5" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b7d0d89c-76ff-4c43-87e1-1290ff7c45d3}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="4faae966-7260-43d3-ae92-efca4c8c38c2">
+    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{f543f122-de6b-42e2-ad09-6f28494b3e44}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="4e3da3af-ee5c-4759-aab6-a01dc2b41ec5">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -6795,22 +6753,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBF2D808-0CB9-47C2-A018-2ECFAB0CA97E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3bb59413-afb5-4b9b-85e8-61d2b74a5666"/>
-    <ds:schemaRef ds:uri="4faae966-7260-43d3-ae92-efca4c8c38c2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E111FA42-621E-434F-A82D-113380E5594C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>